<commit_message>
Refresh from workbook (requested by Jit)
</commit_message>
<xml_diff>
--- a/tools/itinerary.xlsx
+++ b/tools/itinerary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jitwei/Library/Mobile Documents/com~apple~CloudDocs/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4BAEC6-A34F-1948-9AEC-08A088BC0738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1283FF7-42FE-E247-A56C-B529A2C85B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28160" windowHeight="17020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28160" windowHeight="17020" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="1069">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1596" uniqueCount="1075">
   <si>
     <r>
       <rPr>
@@ -8939,9 +8939,6 @@
     <t>18:30–19:45</t>
   </si>
   <si>
-    <t>Dinner</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -12701,12 +12698,6 @@
   </si>
   <si>
     <t>18:00–19:45</t>
-  </si>
-  <si>
-    <t>Farewell dinner — south old town</t>
-  </si>
-  <si>
-    <t>Canal-side dinner near Shiquan/Pingjiang.</t>
   </si>
   <si>
     <t>20:00–21:15</t>
@@ -14556,6 +14547,33 @@
   </si>
   <si>
     <t>¥15–25</t>
+  </si>
+  <si>
+    <t>Farewell dinner — 🦀 HAIRY CRAB: Lao Changmen 老阊门菜馆 (Shantang 山塘街店)</t>
+  </si>
+  <si>
+    <t>Peak 大闸蟹 season — mid-Nov is the 公蟹/蟹膏 window (农历十月). Order 招牌熟醉蟹, 阳澄湖大闸蟹 (market price), 蟹粉豆腐. ~¥100pp, 4.8/5 (small sample, 21 reviews); praised for 物美价廉 &amp; 拒绝料包. ⚠ Queues can exceed 1h at meal times — book or arrive 17:45. ⚠ At ¥100pp the crab is mostly 熟醉蟹, not whole steamed; whole 清蒸 is extra at 时令价. Ask for 现点现炒 蟹粉 and scan the 防伪戒指 QR to verify 阳澄湖 origin. PRESTIGE ALT: 新聚丰菜馆 太监弄店 (est. 1904, 黑珍珠+米其林指南, 清炒蟹粉, ¥215–389) — same lane as today’s lunch, but closes 20:30 and has QC complaints.</t>
+  </si>
+  <si>
+    <t>¥100pp · 山塘街</t>
+  </si>
+  <si>
+    <t>姑苏区山塘街 (老阊门菜馆) · 备选 姑苏区观前街太监弄 (新聚丰)</t>
+  </si>
+  <si>
+    <t>🦀 Crab</t>
+  </si>
+  <si>
+    <t>Lao Changmen 老阊门菜馆 (Day 7 · 山塘街店)</t>
+  </si>
+  <si>
+    <t>姑苏区山塘街 (walkable from the Ritz)</t>
+  </si>
+  <si>
+    <t>HAIRY CRAB 大闸蟹 season pick. 招牌熟醉蟹, 阳澄湖大闸蟹 (时令价), 蟹粉豆腐. 4.8/5 but only 21 reviews; 拒绝料包. Queues &gt;1h at meal times. Prestige alt: 新聚丰菜馆 太监弄店 (1904, 黑珍珠+米其林指南, 清炒蟹粉, ¥215–389, closes 20:30). Lake-view alt: 璞园春舍 on 阳澄湖莲花岛 — boat required, board by 16:30, book 3+ days ahead. Season: 9月下旬–12月; 农历十月 = 公蟹蟹膏. Source: Ctrip reviews via news summary — re-check on Dianping before going.</t>
+  </si>
+  <si>
+    <t>¥100 (蟹另计)</t>
   </si>
 </sst>
 </file>
@@ -16313,7 +16331,7 @@
     </row>
     <row r="4" spans="1:6" ht="30" customHeight="1">
       <c r="A4" s="167" t="s">
-        <v>969</v>
+        <v>966</v>
       </c>
       <c r="B4" s="168"/>
       <c r="C4" s="168"/>
@@ -16366,13 +16384,13 @@
         <v>401</v>
       </c>
       <c r="B7" s="213" t="s">
-        <v>981</v>
+        <v>978</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>412</v>
       </c>
       <c r="D7" s="50" t="s">
-        <v>982</v>
+        <v>979</v>
       </c>
       <c r="E7" s="50" t="s">
         <v>413</v>
@@ -16503,7 +16521,7 @@
     </row>
     <row r="14" spans="1:6" ht="25.5" customHeight="1">
       <c r="A14" s="167" t="s">
-        <v>970</v>
+        <v>967</v>
       </c>
       <c r="B14" s="168"/>
       <c r="C14" s="168"/>
@@ -16616,7 +16634,7 @@
         <v>442</v>
       </c>
       <c r="B20" s="207" t="s">
-        <v>993</v>
+        <v>990</v>
       </c>
       <c r="C20" s="61" t="s">
         <v>465</v>
@@ -16636,7 +16654,7 @@
         <v>442</v>
       </c>
       <c r="B21" s="212" t="s">
-        <v>986</v>
+        <v>983</v>
       </c>
       <c r="C21" s="20" t="s">
         <v>469</v>
@@ -16656,19 +16674,19 @@
         <v>442</v>
       </c>
       <c r="B22" s="212" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>983</v>
+        <v>980</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>984</v>
+        <v>981</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>985</v>
+        <v>982</v>
       </c>
       <c r="F22" s="121" t="s">
-        <v>968</v>
+        <v>965</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="42" customHeight="1">
@@ -16676,7 +16694,7 @@
         <v>442</v>
       </c>
       <c r="B23" s="214" t="s">
-        <v>987</v>
+        <v>984</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>472</v>
@@ -16696,7 +16714,7 @@
         <v>442</v>
       </c>
       <c r="B24" s="207" t="s">
-        <v>988</v>
+        <v>985</v>
       </c>
       <c r="C24" s="61" t="s">
         <v>474</v>
@@ -16716,7 +16734,7 @@
         <v>442</v>
       </c>
       <c r="B25" s="207" t="s">
-        <v>989</v>
+        <v>986</v>
       </c>
       <c r="C25" s="61" t="s">
         <v>478</v>
@@ -16736,7 +16754,7 @@
         <v>442</v>
       </c>
       <c r="B26" s="207" t="s">
-        <v>990</v>
+        <v>987</v>
       </c>
       <c r="C26" s="61" t="s">
         <v>482</v>
@@ -16756,19 +16774,19 @@
         <v>442</v>
       </c>
       <c r="B27" s="207" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C27" s="61" t="s">
-        <v>965</v>
+        <v>962</v>
       </c>
       <c r="D27" s="61" t="s">
-        <v>966</v>
+        <v>963</v>
       </c>
       <c r="E27" s="61" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F27" s="120" t="s">
-        <v>967</v>
+        <v>964</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="42" customHeight="1">
@@ -16776,13 +16794,13 @@
         <v>442</v>
       </c>
       <c r="B28" s="215" t="s">
+        <v>988</v>
+      </c>
+      <c r="C28" s="36" t="s">
         <v>991</v>
       </c>
-      <c r="C28" s="36" t="s">
-        <v>994</v>
-      </c>
       <c r="D28" s="36" t="s">
-        <v>995</v>
+        <v>992</v>
       </c>
       <c r="E28" s="36" t="s">
         <v>61</v>
@@ -16796,13 +16814,13 @@
         <v>442</v>
       </c>
       <c r="B29" s="209" t="s">
-        <v>992</v>
+        <v>989</v>
       </c>
       <c r="C29" s="33" t="s">
         <v>486</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="E29" s="33" t="s">
         <v>487</v>
@@ -16816,19 +16834,19 @@
         <v>442</v>
       </c>
       <c r="B30" s="218" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C30" s="61" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D30" s="61" t="s">
+        <v>1036</v>
+      </c>
+      <c r="E30" s="61" t="s">
+        <v>1037</v>
+      </c>
+      <c r="F30" s="120" t="s">
         <v>1038</v>
-      </c>
-      <c r="D30" s="61" t="s">
-        <v>1039</v>
-      </c>
-      <c r="E30" s="61" t="s">
-        <v>1040</v>
-      </c>
-      <c r="F30" s="120" t="s">
-        <v>1041</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="42" customHeight="1">
@@ -16836,19 +16854,19 @@
         <v>442</v>
       </c>
       <c r="B31" s="218" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C31" s="61" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D31" s="61" t="s">
+        <v>1040</v>
+      </c>
+      <c r="E31" s="61" t="s">
+        <v>1041</v>
+      </c>
+      <c r="F31" s="120" t="s">
         <v>1042</v>
-      </c>
-      <c r="D31" s="61" t="s">
-        <v>1043</v>
-      </c>
-      <c r="E31" s="61" t="s">
-        <v>1044</v>
-      </c>
-      <c r="F31" s="120" t="s">
-        <v>1045</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="56" customHeight="1">
@@ -16856,19 +16874,19 @@
         <v>442</v>
       </c>
       <c r="B32" s="218" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C32" s="61" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D32" s="61" t="s">
+        <v>1051</v>
+      </c>
+      <c r="E32" s="61" t="s">
+        <v>1052</v>
+      </c>
+      <c r="F32" s="120" t="s">
         <v>1053</v>
-      </c>
-      <c r="D32" s="61" t="s">
-        <v>1054</v>
-      </c>
-      <c r="E32" s="61" t="s">
-        <v>1055</v>
-      </c>
-      <c r="F32" s="120" t="s">
-        <v>1056</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="25.5" customHeight="1">
@@ -16876,19 +16894,19 @@
         <v>442</v>
       </c>
       <c r="B33" s="57" t="s">
+        <v>936</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>937</v>
+      </c>
+      <c r="D33" s="33" t="s">
+        <v>938</v>
+      </c>
+      <c r="E33" s="33" t="s">
         <v>939</v>
       </c>
-      <c r="C33" s="33" t="s">
+      <c r="F33" s="117" t="s">
         <v>940</v>
-      </c>
-      <c r="D33" s="33" t="s">
-        <v>941</v>
-      </c>
-      <c r="E33" s="33" t="s">
-        <v>942</v>
-      </c>
-      <c r="F33" s="117" t="s">
-        <v>943</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="30" customHeight="1">
@@ -16896,7 +16914,7 @@
         <v>442</v>
       </c>
       <c r="B34" s="64" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
       <c r="C34" s="36" t="s">
         <v>488</v>
@@ -16916,7 +16934,7 @@
         <v>442</v>
       </c>
       <c r="B35" s="151" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="C35" s="10" t="s">
         <v>493</v>
@@ -16931,7 +16949,7 @@
     </row>
     <row r="36" spans="1:6" ht="25.5" customHeight="1">
       <c r="A36" s="167" t="s">
-        <v>971</v>
+        <v>968</v>
       </c>
       <c r="B36" s="168"/>
       <c r="C36" s="168"/>
@@ -16964,19 +16982,19 @@
         <v>494</v>
       </c>
       <c r="B38" s="209" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C38" s="33" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D38" s="33" t="s">
+        <v>1059</v>
+      </c>
+      <c r="E38" s="35" t="s">
+        <v>1060</v>
+      </c>
+      <c r="F38" s="117" t="s">
         <v>1061</v>
-      </c>
-      <c r="D38" s="33" t="s">
-        <v>1062</v>
-      </c>
-      <c r="E38" s="35" t="s">
-        <v>1063</v>
-      </c>
-      <c r="F38" s="117" t="s">
-        <v>1064</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="30" customHeight="1">
@@ -17104,19 +17122,19 @@
         <v>494</v>
       </c>
       <c r="B45" s="89" t="s">
+        <v>897</v>
+      </c>
+      <c r="C45" s="90" t="s">
+        <v>898</v>
+      </c>
+      <c r="D45" s="90" t="s">
+        <v>899</v>
+      </c>
+      <c r="E45" s="90" t="s">
         <v>900</v>
       </c>
-      <c r="C45" s="90" t="s">
+      <c r="F45" s="123" t="s">
         <v>901</v>
-      </c>
-      <c r="D45" s="90" t="s">
-        <v>902</v>
-      </c>
-      <c r="E45" s="90" t="s">
-        <v>903</v>
-      </c>
-      <c r="F45" s="123" t="s">
-        <v>904</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="25.5" customHeight="1">
@@ -17124,7 +17142,7 @@
         <v>494</v>
       </c>
       <c r="B46" s="57" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C46" s="33" t="s">
         <v>523</v>
@@ -17144,19 +17162,19 @@
         <v>494</v>
       </c>
       <c r="B47" s="209" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>962</v>
+        <v>959</v>
       </c>
       <c r="D47" s="33" t="s">
-        <v>963</v>
+        <v>960</v>
       </c>
       <c r="E47" s="35" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F47" s="117" t="s">
-        <v>964</v>
+        <v>961</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="42" customHeight="1">
@@ -17164,7 +17182,7 @@
         <v>494</v>
       </c>
       <c r="B48" s="63" t="s">
-        <v>922</v>
+        <v>919</v>
       </c>
       <c r="C48" s="20" t="s">
         <v>527</v>
@@ -17184,13 +17202,13 @@
         <v>494</v>
       </c>
       <c r="B49" s="207" t="s">
-        <v>996</v>
+        <v>993</v>
       </c>
       <c r="C49" s="61" t="s">
         <v>530</v>
       </c>
       <c r="D49" s="61" t="s">
-        <v>997</v>
+        <v>994</v>
       </c>
       <c r="E49" s="61" t="s">
         <v>531</v>
@@ -17204,16 +17222,16 @@
         <v>494</v>
       </c>
       <c r="B50" s="210" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C50" s="39" t="s">
         <v>533</v>
       </c>
       <c r="D50" s="39" t="s">
-        <v>998</v>
+        <v>995</v>
       </c>
       <c r="E50" s="39" t="s">
-        <v>999</v>
+        <v>996</v>
       </c>
       <c r="F50" s="118" t="s">
         <v>535</v>
@@ -17224,19 +17242,19 @@
         <v>494</v>
       </c>
       <c r="B51" s="53" t="s">
+        <v>997</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>998</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>999</v>
+      </c>
+      <c r="E51" s="5" t="s">
         <v>1000</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="F51" s="86" t="s">
         <v>1001</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>1002</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>1003</v>
-      </c>
-      <c r="F51" s="86" t="s">
-        <v>1004</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="42" customHeight="1">
@@ -17244,19 +17262,19 @@
         <v>494</v>
       </c>
       <c r="B52" s="214" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>1004</v>
+      </c>
+      <c r="E52" s="5" t="s">
         <v>1005</v>
       </c>
-      <c r="C52" s="5" t="s">
-        <v>1006</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>1007</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>1008</v>
-      </c>
       <c r="F52" s="86" t="s">
-        <v>1004</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="30" customHeight="1">
@@ -17264,13 +17282,13 @@
         <v>494</v>
       </c>
       <c r="B53" s="151" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>1009</v>
+        <v>1006</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>441</v>
@@ -17284,16 +17302,16 @@
         <v>494</v>
       </c>
       <c r="B54" s="65" t="s">
+        <v>538</v>
+      </c>
+      <c r="C54" s="42" t="s">
         <v>539</v>
       </c>
-      <c r="C54" s="42" t="s">
+      <c r="D54" s="42" t="s">
         <v>540</v>
       </c>
-      <c r="D54" s="42" t="s">
+      <c r="E54" s="42" t="s">
         <v>541</v>
-      </c>
-      <c r="E54" s="42" t="s">
-        <v>542</v>
       </c>
       <c r="F54" s="124" t="s">
         <v>312</v>
@@ -17304,19 +17322,19 @@
         <v>494</v>
       </c>
       <c r="B55" s="58" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C55" s="39" t="s">
+        <v>542</v>
+      </c>
+      <c r="D55" s="39" t="s">
         <v>543</v>
       </c>
-      <c r="D55" s="39" t="s">
+      <c r="E55" s="39" t="s">
+        <v>541</v>
+      </c>
+      <c r="F55" s="118" t="s">
         <v>544</v>
-      </c>
-      <c r="E55" s="39" t="s">
-        <v>542</v>
-      </c>
-      <c r="F55" s="118" t="s">
-        <v>545</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="25.5" customHeight="1">
@@ -17324,24 +17342,24 @@
         <v>494</v>
       </c>
       <c r="B56" s="210" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C56" s="39" t="s">
+        <v>955</v>
+      </c>
+      <c r="D56" s="211" t="s">
+        <v>956</v>
+      </c>
+      <c r="E56" s="39" t="s">
+        <v>957</v>
+      </c>
+      <c r="F56" s="118" t="s">
         <v>958</v>
-      </c>
-      <c r="D56" s="211" t="s">
-        <v>959</v>
-      </c>
-      <c r="E56" s="39" t="s">
-        <v>960</v>
-      </c>
-      <c r="F56" s="118" t="s">
-        <v>961</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="25.5" customHeight="1">
       <c r="A57" s="152" t="s">
-        <v>978</v>
+        <v>975</v>
       </c>
       <c r="B57" s="153"/>
       <c r="C57" s="153"/>
@@ -17351,19 +17369,19 @@
     </row>
     <row r="58" spans="1:6" ht="45" customHeight="1">
       <c r="A58" s="101" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B58" s="56" t="s">
         <v>495</v>
       </c>
       <c r="C58" s="10" t="s">
+        <v>546</v>
+      </c>
+      <c r="D58" s="10" t="s">
         <v>547</v>
       </c>
-      <c r="D58" s="10" t="s">
+      <c r="E58" s="10" t="s">
         <v>548</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>549</v>
       </c>
       <c r="F58" s="116" t="s">
         <v>28</v>
@@ -17371,76 +17389,76 @@
     </row>
     <row r="59" spans="1:6" ht="25.5" customHeight="1">
       <c r="A59" s="100" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B59" s="55" t="s">
+        <v>549</v>
+      </c>
+      <c r="C59" s="50" t="s">
         <v>550</v>
       </c>
-      <c r="C59" s="50" t="s">
+      <c r="D59" s="50" t="s">
         <v>551</v>
       </c>
-      <c r="D59" s="50" t="s">
+      <c r="E59" s="50" t="s">
         <v>552</v>
       </c>
-      <c r="E59" s="50" t="s">
+      <c r="F59" s="115" t="s">
         <v>553</v>
-      </c>
-      <c r="F59" s="115" t="s">
-        <v>554</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="30" customHeight="1">
       <c r="A60" s="100" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B60" s="55" t="s">
+        <v>554</v>
+      </c>
+      <c r="C60" s="50" t="s">
         <v>555</v>
       </c>
-      <c r="C60" s="50" t="s">
+      <c r="D60" s="50" t="s">
         <v>556</v>
       </c>
-      <c r="D60" s="50" t="s">
+      <c r="E60" s="50" t="s">
         <v>557</v>
       </c>
-      <c r="E60" s="50" t="s">
+      <c r="F60" s="115" t="s">
         <v>558</v>
-      </c>
-      <c r="F60" s="115" t="s">
-        <v>559</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="30" customHeight="1">
       <c r="A61" s="101" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B61" s="56" t="s">
+        <v>559</v>
+      </c>
+      <c r="C61" s="10" t="s">
         <v>560</v>
       </c>
-      <c r="C61" s="10" t="s">
+      <c r="D61" s="10" t="s">
         <v>561</v>
-      </c>
-      <c r="D61" s="10" t="s">
-        <v>562</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>423</v>
       </c>
       <c r="F61" s="116" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="25.5" customHeight="1">
       <c r="A62" s="99" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B62" s="54" t="s">
+        <v>563</v>
+      </c>
+      <c r="C62" s="15" t="s">
         <v>564</v>
       </c>
-      <c r="C62" s="15" t="s">
+      <c r="D62" s="25" t="s">
         <v>565</v>
-      </c>
-      <c r="D62" s="25" t="s">
-        <v>566</v>
       </c>
       <c r="E62" s="15" t="s">
         <v>166</v>
@@ -17451,16 +17469,16 @@
     </row>
     <row r="63" spans="1:6" ht="21.75" customHeight="1">
       <c r="A63" s="105" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B63" s="60" t="s">
+        <v>566</v>
+      </c>
+      <c r="C63" s="61" t="s">
         <v>567</v>
       </c>
-      <c r="C63" s="61" t="s">
+      <c r="D63" s="61" t="s">
         <v>568</v>
-      </c>
-      <c r="D63" s="61" t="s">
-        <v>569</v>
       </c>
       <c r="E63" s="61" t="s">
         <v>505</v>
@@ -17471,165 +17489,165 @@
     </row>
     <row r="64" spans="1:6" ht="25.5" customHeight="1">
       <c r="A64" s="105" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B64" s="60" t="s">
+        <v>569</v>
+      </c>
+      <c r="C64" s="61" t="s">
         <v>570</v>
       </c>
-      <c r="C64" s="61" t="s">
+      <c r="D64" s="61" t="s">
         <v>571</v>
       </c>
-      <c r="D64" s="61" t="s">
+      <c r="E64" s="61" t="s">
         <v>572</v>
       </c>
-      <c r="E64" s="61" t="s">
+      <c r="F64" s="120" t="s">
         <v>573</v>
-      </c>
-      <c r="F64" s="120" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="25.5" customHeight="1">
       <c r="A65" s="106" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B65" s="63" t="s">
+        <v>574</v>
+      </c>
+      <c r="C65" s="20" t="s">
         <v>575</v>
       </c>
-      <c r="C65" s="20" t="s">
+      <c r="D65" s="20" t="s">
         <v>576</v>
       </c>
-      <c r="D65" s="20" t="s">
+      <c r="E65" s="20" t="s">
         <v>577</v>
       </c>
-      <c r="E65" s="20" t="s">
+      <c r="F65" s="121" t="s">
         <v>578</v>
-      </c>
-      <c r="F65" s="121" t="s">
-        <v>579</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="30" customHeight="1">
       <c r="A66" s="105" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B66" s="60" t="s">
+        <v>579</v>
+      </c>
+      <c r="C66" s="61" t="s">
         <v>580</v>
       </c>
-      <c r="C66" s="61" t="s">
+      <c r="D66" s="61" t="s">
         <v>581</v>
       </c>
-      <c r="D66" s="61" t="s">
+      <c r="E66" s="61" t="s">
+        <v>572</v>
+      </c>
+      <c r="F66" s="120" t="s">
         <v>582</v>
-      </c>
-      <c r="E66" s="61" t="s">
-        <v>573</v>
-      </c>
-      <c r="F66" s="120" t="s">
-        <v>583</v>
       </c>
     </row>
     <row r="67" spans="1:6" ht="30" customHeight="1">
       <c r="A67" s="110" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B67" s="91" t="s">
-        <v>923</v>
+        <v>920</v>
       </c>
       <c r="C67" s="92" t="s">
+        <v>902</v>
+      </c>
+      <c r="D67" s="92" t="s">
+        <v>903</v>
+      </c>
+      <c r="E67" s="92" t="s">
+        <v>904</v>
+      </c>
+      <c r="F67" s="125" t="s">
         <v>905</v>
-      </c>
-      <c r="D67" s="92" t="s">
-        <v>906</v>
-      </c>
-      <c r="E67" s="92" t="s">
-        <v>907</v>
-      </c>
-      <c r="F67" s="125" t="s">
-        <v>908</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="30" customHeight="1">
       <c r="A68" s="105" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B68" s="60" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C68" s="61" t="s">
+        <v>583</v>
+      </c>
+      <c r="D68" s="61" t="s">
         <v>584</v>
       </c>
-      <c r="D68" s="61" t="s">
+      <c r="E68" s="61" t="s">
         <v>585</v>
       </c>
-      <c r="E68" s="61" t="s">
+      <c r="F68" s="120" t="s">
         <v>586</v>
-      </c>
-      <c r="F68" s="120" t="s">
-        <v>587</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="25.5" customHeight="1">
       <c r="A69" s="107" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B69" s="64" t="s">
-        <v>924</v>
+        <v>921</v>
       </c>
       <c r="C69" s="36" t="s">
+        <v>588</v>
+      </c>
+      <c r="D69" s="36" t="s">
         <v>589</v>
       </c>
-      <c r="D69" s="36" t="s">
+      <c r="E69" s="36" t="s">
         <v>590</v>
       </c>
-      <c r="E69" s="36" t="s">
+      <c r="F69" s="122" t="s">
         <v>591</v>
-      </c>
-      <c r="F69" s="122" t="s">
-        <v>592</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="25.5" customHeight="1">
       <c r="A70" s="109" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B70" s="65" t="s">
-        <v>925</v>
+        <v>922</v>
       </c>
       <c r="C70" s="42" t="s">
+        <v>592</v>
+      </c>
+      <c r="D70" s="44" t="s">
         <v>593</v>
       </c>
-      <c r="D70" s="44" t="s">
+      <c r="E70" s="42" t="s">
         <v>594</v>
       </c>
-      <c r="E70" s="42" t="s">
+      <c r="F70" s="124" t="s">
         <v>595</v>
-      </c>
-      <c r="F70" s="124" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="30" customHeight="1">
       <c r="A71" s="101" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B71" s="128" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="D71" s="10"/>
       <c r="E71" s="10" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="F71" s="116" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="30" customHeight="1">
       <c r="A72" s="152" t="s">
-        <v>972</v>
+        <v>969</v>
       </c>
       <c r="B72" s="153"/>
       <c r="C72" s="153"/>
@@ -17639,16 +17657,16 @@
     </row>
     <row r="73" spans="1:6" ht="30" customHeight="1">
       <c r="A73" s="101" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B73" s="56" t="s">
         <v>495</v>
       </c>
       <c r="C73" s="10" t="s">
+        <v>600</v>
+      </c>
+      <c r="D73" s="10" t="s">
         <v>601</v>
-      </c>
-      <c r="D73" s="10" t="s">
-        <v>602</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>20</v>
@@ -17659,219 +17677,219 @@
     </row>
     <row r="74" spans="1:6" ht="25.5" customHeight="1">
       <c r="A74" s="105" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B74" s="60" t="s">
+        <v>602</v>
+      </c>
+      <c r="C74" s="61" t="s">
         <v>603</v>
       </c>
-      <c r="C74" s="61" t="s">
+      <c r="D74" s="62" t="s">
         <v>604</v>
       </c>
-      <c r="D74" s="62" t="s">
+      <c r="E74" s="61" t="s">
         <v>605</v>
       </c>
-      <c r="E74" s="61" t="s">
+      <c r="F74" s="120" t="s">
         <v>606</v>
-      </c>
-      <c r="F74" s="120" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="30" customHeight="1">
       <c r="A75" s="108" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B75" s="89" t="s">
+        <v>906</v>
+      </c>
+      <c r="C75" s="90" t="s">
+        <v>907</v>
+      </c>
+      <c r="D75" s="90" t="s">
+        <v>908</v>
+      </c>
+      <c r="E75" s="90" t="s">
         <v>909</v>
       </c>
-      <c r="C75" s="90" t="s">
+      <c r="F75" s="123" t="s">
         <v>910</v>
-      </c>
-      <c r="D75" s="90" t="s">
-        <v>911</v>
-      </c>
-      <c r="E75" s="90" t="s">
-        <v>912</v>
-      </c>
-      <c r="F75" s="123" t="s">
-        <v>913</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="30" customHeight="1">
       <c r="A76" s="103" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B76" s="58" t="s">
-        <v>926</v>
+        <v>923</v>
       </c>
       <c r="C76" s="39" t="s">
+        <v>607</v>
+      </c>
+      <c r="D76" s="39" t="s">
         <v>608</v>
       </c>
-      <c r="D76" s="39" t="s">
+      <c r="E76" s="39" t="s">
         <v>609</v>
       </c>
-      <c r="E76" s="39" t="s">
+      <c r="F76" s="118" t="s">
         <v>610</v>
-      </c>
-      <c r="F76" s="118" t="s">
-        <v>611</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="42" customHeight="1">
       <c r="A77" s="104" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B77" s="59" t="s">
         <v>464</v>
       </c>
       <c r="C77" s="47" t="s">
+        <v>611</v>
+      </c>
+      <c r="D77" s="47" t="s">
         <v>612</v>
       </c>
-      <c r="D77" s="47" t="s">
+      <c r="E77" s="47" t="s">
         <v>613</v>
       </c>
-      <c r="E77" s="47" t="s">
+      <c r="F77" s="119" t="s">
         <v>614</v>
-      </c>
-      <c r="F77" s="119" t="s">
-        <v>615</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="25.5" customHeight="1">
       <c r="A78" s="105" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B78" s="60" t="s">
+        <v>615</v>
+      </c>
+      <c r="C78" s="61" t="s">
         <v>616</v>
       </c>
-      <c r="C78" s="61" t="s">
+      <c r="D78" s="61" t="s">
         <v>617</v>
       </c>
-      <c r="D78" s="61" t="s">
+      <c r="E78" s="61" t="s">
         <v>618</v>
       </c>
-      <c r="E78" s="61" t="s">
+      <c r="F78" s="120" t="s">
         <v>619</v>
-      </c>
-      <c r="F78" s="120" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="79" spans="1:6" ht="30" customHeight="1">
       <c r="A79" s="98" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B79" s="53" t="s">
+        <v>620</v>
+      </c>
+      <c r="C79" s="5" t="s">
         <v>621</v>
       </c>
-      <c r="C79" s="5" t="s">
+      <c r="D79" s="5" t="s">
         <v>622</v>
       </c>
-      <c r="D79" s="5" t="s">
+      <c r="E79" s="5" t="s">
         <v>623</v>
       </c>
-      <c r="E79" s="5" t="s">
+      <c r="F79" s="86" t="s">
         <v>624</v>
-      </c>
-      <c r="F79" s="86" t="s">
-        <v>625</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="30" customHeight="1">
       <c r="A80" s="103" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B80" s="58" t="s">
+        <v>625</v>
+      </c>
+      <c r="C80" s="39" t="s">
         <v>626</v>
       </c>
-      <c r="C80" s="39" t="s">
+      <c r="D80" s="39" t="s">
         <v>627</v>
       </c>
-      <c r="D80" s="39" t="s">
+      <c r="E80" s="39" t="s">
         <v>628</v>
       </c>
-      <c r="E80" s="39" t="s">
+      <c r="F80" s="118" t="s">
         <v>629</v>
-      </c>
-      <c r="F80" s="118" t="s">
-        <v>630</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="42" customHeight="1">
       <c r="A81" s="105" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B81" s="60" t="s">
+        <v>630</v>
+      </c>
+      <c r="C81" s="61" t="s">
         <v>631</v>
       </c>
-      <c r="C81" s="61" t="s">
+      <c r="D81" s="61" t="s">
         <v>632</v>
       </c>
-      <c r="D81" s="61" t="s">
+      <c r="E81" s="61" t="s">
         <v>633</v>
       </c>
-      <c r="E81" s="61" t="s">
+      <c r="F81" s="120" t="s">
         <v>634</v>
-      </c>
-      <c r="F81" s="120" t="s">
-        <v>635</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="30" customHeight="1">
       <c r="A82" s="104" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B82" s="59" t="s">
+        <v>635</v>
+      </c>
+      <c r="C82" s="47" t="s">
         <v>636</v>
       </c>
-      <c r="C82" s="47" t="s">
+      <c r="D82" s="47" t="s">
         <v>637</v>
       </c>
-      <c r="D82" s="47" t="s">
+      <c r="E82" s="47" t="s">
+        <v>628</v>
+      </c>
+      <c r="F82" s="119" t="s">
         <v>638</v>
-      </c>
-      <c r="E82" s="47" t="s">
-        <v>629</v>
-      </c>
-      <c r="F82" s="119" t="s">
-        <v>639</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="21.75" customHeight="1">
       <c r="A83" s="106" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B83" s="63" t="s">
+        <v>639</v>
+      </c>
+      <c r="C83" s="20" t="s">
         <v>640</v>
       </c>
-      <c r="C83" s="20" t="s">
+      <c r="D83" s="20" t="s">
         <v>641</v>
       </c>
-      <c r="D83" s="20" t="s">
+      <c r="E83" s="20" t="s">
         <v>642</v>
       </c>
-      <c r="E83" s="20" t="s">
+      <c r="F83" s="121" t="s">
         <v>643</v>
-      </c>
-      <c r="F83" s="121" t="s">
-        <v>644</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="42" customHeight="1">
       <c r="A84" s="102" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B84" s="57" t="s">
+        <v>644</v>
+      </c>
+      <c r="C84" s="33" t="s">
         <v>645</v>
       </c>
-      <c r="C84" s="33" t="s">
+      <c r="D84" s="33" t="s">
         <v>646</v>
       </c>
-      <c r="D84" s="33" t="s">
+      <c r="E84" s="33" t="s">
         <v>647</v>
-      </c>
-      <c r="E84" s="33" t="s">
-        <v>648</v>
       </c>
       <c r="F84" s="117" t="s">
         <v>33</v>
@@ -17879,36 +17897,36 @@
     </row>
     <row r="85" spans="1:6" ht="25.5" customHeight="1">
       <c r="A85" s="102" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B85" s="209" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C85" s="33" t="s">
-        <v>955</v>
+        <v>952</v>
       </c>
       <c r="D85" s="33" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
       <c r="E85" s="33" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F85" s="117" t="s">
-        <v>957</v>
+        <v>954</v>
       </c>
     </row>
     <row r="86" spans="1:6" ht="25.5" customHeight="1">
       <c r="A86" s="107" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B86" s="64" t="s">
         <v>536</v>
       </c>
       <c r="C86" s="36" t="s">
+        <v>648</v>
+      </c>
+      <c r="D86" s="36" t="s">
         <v>649</v>
-      </c>
-      <c r="D86" s="36" t="s">
-        <v>650</v>
       </c>
       <c r="E86" s="36" t="s">
         <v>209</v>
@@ -17919,16 +17937,16 @@
     </row>
     <row r="87" spans="1:6" ht="30" customHeight="1">
       <c r="A87" s="101" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B87" s="56" t="s">
+        <v>650</v>
+      </c>
+      <c r="C87" s="10" t="s">
         <v>651</v>
       </c>
-      <c r="C87" s="10" t="s">
+      <c r="D87" s="10" t="s">
         <v>652</v>
-      </c>
-      <c r="D87" s="10" t="s">
-        <v>653</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>534</v>
@@ -17939,127 +17957,127 @@
     </row>
     <row r="88" spans="1:6" ht="25.5" customHeight="1">
       <c r="A88" s="101" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B88" s="56" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C88" s="10" t="s">
+        <v>653</v>
+      </c>
+      <c r="D88" s="10" t="s">
         <v>654</v>
       </c>
-      <c r="D88" s="10" t="s">
-        <v>655</v>
-      </c>
       <c r="E88" s="10" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="F88" s="116" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="89" spans="1:6" ht="42" customHeight="1">
       <c r="A89" s="103" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B89" s="58" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C89" s="39" t="s">
+        <v>655</v>
+      </c>
+      <c r="D89" s="39" t="s">
         <v>656</v>
       </c>
-      <c r="D89" s="39" t="s">
+      <c r="E89" s="39" t="s">
+        <v>541</v>
+      </c>
+      <c r="F89" s="118" t="s">
         <v>657</v>
-      </c>
-      <c r="E89" s="39" t="s">
-        <v>542</v>
-      </c>
-      <c r="F89" s="118" t="s">
-        <v>658</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="30" customHeight="1">
       <c r="A90" s="103" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B90" s="58" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C90" s="39" t="s">
+        <v>658</v>
+      </c>
+      <c r="D90" s="39" t="s">
         <v>659</v>
       </c>
-      <c r="D90" s="39" t="s">
+      <c r="E90" s="39" t="s">
+        <v>541</v>
+      </c>
+      <c r="F90" s="118" t="s">
         <v>660</v>
-      </c>
-      <c r="E90" s="39" t="s">
-        <v>542</v>
-      </c>
-      <c r="F90" s="118" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="91" spans="1:6" ht="25.5" customHeight="1">
       <c r="A91" s="103" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B91" s="58" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C91" s="39" t="s">
+        <v>661</v>
+      </c>
+      <c r="D91" s="39" t="s">
         <v>662</v>
       </c>
-      <c r="D91" s="39" t="s">
+      <c r="E91" s="39" t="s">
+        <v>541</v>
+      </c>
+      <c r="F91" s="118" t="s">
         <v>663</v>
-      </c>
-      <c r="E91" s="39" t="s">
-        <v>542</v>
-      </c>
-      <c r="F91" s="118" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="92" spans="1:6" ht="25.5" customHeight="1">
       <c r="A92" s="108" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B92" s="89" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C92" s="90" t="s">
+        <v>911</v>
+      </c>
+      <c r="D92" s="95" t="s">
+        <v>912</v>
+      </c>
+      <c r="E92" s="90" t="s">
+        <v>913</v>
+      </c>
+      <c r="F92" s="123" t="s">
         <v>914</v>
-      </c>
-      <c r="D92" s="95" t="s">
-        <v>915</v>
-      </c>
-      <c r="E92" s="90" t="s">
-        <v>916</v>
-      </c>
-      <c r="F92" s="123" t="s">
-        <v>917</v>
       </c>
     </row>
     <row r="93" spans="1:6" ht="30" customHeight="1">
       <c r="A93" s="108" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B93" s="208" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C93" s="90" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
       <c r="D93" s="95" t="s">
-        <v>953</v>
+        <v>950</v>
       </c>
       <c r="E93" s="90" t="s">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="F93" s="123" t="s">
-        <v>954</v>
+        <v>951</v>
       </c>
     </row>
     <row r="94" spans="1:6" ht="30" customHeight="1">
       <c r="A94" s="155" t="s">
-        <v>979</v>
+        <v>976</v>
       </c>
       <c r="B94" s="156"/>
       <c r="C94" s="156"/>
@@ -18069,17 +18087,17 @@
     </row>
     <row r="95" spans="1:6" ht="42" customHeight="1">
       <c r="A95" s="101" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B95" s="56" t="s">
         <v>495</v>
       </c>
       <c r="C95" s="10" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D95" s="10"/>
       <c r="E95" s="10" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F95" s="116" t="s">
         <v>33</v>
@@ -18087,76 +18105,76 @@
     </row>
     <row r="96" spans="1:6" ht="25.5" customHeight="1">
       <c r="A96" s="100" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B96" s="55" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C96" s="50" t="s">
+        <v>666</v>
+      </c>
+      <c r="D96" s="50" t="s">
         <v>667</v>
       </c>
-      <c r="D96" s="50" t="s">
+      <c r="E96" s="50" t="s">
+        <v>552</v>
+      </c>
+      <c r="F96" s="115" t="s">
         <v>668</v>
-      </c>
-      <c r="E96" s="50" t="s">
-        <v>553</v>
-      </c>
-      <c r="F96" s="115" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="97" spans="1:6" ht="45" customHeight="1">
       <c r="A97" s="100" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B97" s="55" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C97" s="50" t="s">
+        <v>669</v>
+      </c>
+      <c r="D97" s="50" t="s">
         <v>670</v>
       </c>
-      <c r="D97" s="50" t="s">
+      <c r="E97" s="50" t="s">
+        <v>557</v>
+      </c>
+      <c r="F97" s="115" t="s">
         <v>671</v>
-      </c>
-      <c r="E97" s="50" t="s">
-        <v>558</v>
-      </c>
-      <c r="F97" s="115" t="s">
-        <v>672</v>
       </c>
     </row>
     <row r="98" spans="1:6" ht="30" customHeight="1">
       <c r="A98" s="101" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B98" s="56" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C98" s="10" t="s">
+        <v>672</v>
+      </c>
+      <c r="D98" s="10" t="s">
         <v>673</v>
       </c>
-      <c r="D98" s="10" t="s">
+      <c r="E98" s="10" t="s">
         <v>674</v>
       </c>
-      <c r="E98" s="10" t="s">
+      <c r="F98" s="116" t="s">
         <v>675</v>
-      </c>
-      <c r="F98" s="116" t="s">
-        <v>676</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="21.75" customHeight="1">
       <c r="A99" s="99" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B99" s="54" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C99" s="15" t="s">
+        <v>676</v>
+      </c>
+      <c r="D99" s="15" t="s">
         <v>677</v>
-      </c>
-      <c r="D99" s="15" t="s">
-        <v>678</v>
       </c>
       <c r="E99" s="15" t="s">
         <v>219</v>
@@ -18167,79 +18185,79 @@
     </row>
     <row r="100" spans="1:6" ht="25.5" customHeight="1">
       <c r="A100" s="105" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B100" s="60" t="s">
+        <v>678</v>
+      </c>
+      <c r="C100" s="61" t="s">
         <v>679</v>
       </c>
-      <c r="C100" s="61" t="s">
+      <c r="D100" s="61" t="s">
         <v>680</v>
       </c>
-      <c r="D100" s="61" t="s">
+      <c r="E100" s="61" t="s">
         <v>681</v>
       </c>
-      <c r="E100" s="61" t="s">
+      <c r="F100" s="120" t="s">
         <v>682</v>
-      </c>
-      <c r="F100" s="120" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="101" spans="1:6" ht="42" customHeight="1">
       <c r="A101" s="105" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B101" s="60" t="s">
+        <v>683</v>
+      </c>
+      <c r="C101" s="61" t="s">
         <v>684</v>
       </c>
-      <c r="C101" s="61" t="s">
+      <c r="D101" s="61" t="s">
         <v>685</v>
       </c>
-      <c r="D101" s="61" t="s">
+      <c r="E101" s="61" t="s">
+        <v>605</v>
+      </c>
+      <c r="F101" s="120" t="s">
         <v>686</v>
-      </c>
-      <c r="E101" s="61" t="s">
-        <v>606</v>
-      </c>
-      <c r="F101" s="120" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="30" customHeight="1">
       <c r="A102" s="105" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B102" s="60" t="s">
+        <v>687</v>
+      </c>
+      <c r="C102" s="61" t="s">
         <v>688</v>
       </c>
-      <c r="C102" s="61" t="s">
+      <c r="D102" s="61" t="s">
         <v>689</v>
       </c>
-      <c r="D102" s="61" t="s">
+      <c r="E102" s="61" t="s">
         <v>690</v>
       </c>
-      <c r="E102" s="61" t="s">
+      <c r="F102" s="120" t="s">
         <v>691</v>
-      </c>
-      <c r="F102" s="120" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="45" customHeight="1">
       <c r="A103" s="106" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B103" s="63" t="s">
+        <v>692</v>
+      </c>
+      <c r="C103" s="20" t="s">
         <v>693</v>
       </c>
-      <c r="C103" s="20" t="s">
+      <c r="D103" s="20" t="s">
         <v>694</v>
       </c>
-      <c r="D103" s="20" t="s">
+      <c r="E103" s="20" t="s">
         <v>695</v>
-      </c>
-      <c r="E103" s="20" t="s">
-        <v>696</v>
       </c>
       <c r="F103" s="121" t="s">
         <v>271</v>
@@ -18247,16 +18265,16 @@
     </row>
     <row r="104" spans="1:6" ht="25.5" customHeight="1">
       <c r="A104" s="105" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B104" s="60" t="s">
+        <v>696</v>
+      </c>
+      <c r="C104" s="61" t="s">
         <v>697</v>
       </c>
-      <c r="C104" s="61" t="s">
+      <c r="D104" s="61" t="s">
         <v>698</v>
-      </c>
-      <c r="D104" s="61" t="s">
-        <v>699</v>
       </c>
       <c r="E104" s="61" t="s">
         <v>111</v>
@@ -18267,19 +18285,19 @@
     </row>
     <row r="105" spans="1:6" ht="42" customHeight="1">
       <c r="A105" s="105" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B105" s="207" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C105" s="61" t="s">
-        <v>950</v>
+        <v>947</v>
       </c>
       <c r="D105" s="61" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="E105" s="61" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F105" s="120" t="s">
         <v>271</v>
@@ -18287,39 +18305,39 @@
     </row>
     <row r="106" spans="1:6" ht="42" customHeight="1">
       <c r="A106" s="109" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B106" s="65" t="s">
+        <v>699</v>
+      </c>
+      <c r="C106" s="42" t="s">
         <v>700</v>
       </c>
-      <c r="C106" s="42" t="s">
+      <c r="D106" s="42" t="s">
         <v>701</v>
       </c>
-      <c r="D106" s="42" t="s">
+      <c r="E106" s="42" t="s">
         <v>702</v>
       </c>
-      <c r="E106" s="42" t="s">
+      <c r="F106" s="124" t="s">
         <v>703</v>
-      </c>
-      <c r="F106" s="124" t="s">
-        <v>704</v>
       </c>
     </row>
     <row r="107" spans="1:6" ht="30" customHeight="1">
       <c r="A107" s="111" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B107" s="93" t="s">
+        <v>915</v>
+      </c>
+      <c r="C107" s="94" t="s">
+        <v>916</v>
+      </c>
+      <c r="D107" s="94" t="s">
+        <v>917</v>
+      </c>
+      <c r="E107" s="94" t="s">
         <v>918</v>
-      </c>
-      <c r="C107" s="94" t="s">
-        <v>919</v>
-      </c>
-      <c r="D107" s="94" t="s">
-        <v>920</v>
-      </c>
-      <c r="E107" s="94" t="s">
-        <v>921</v>
       </c>
       <c r="F107" s="126" t="s">
         <v>278</v>
@@ -18327,34 +18345,34 @@
     </row>
     <row r="108" spans="1:6" ht="25.5" customHeight="1">
       <c r="A108" s="101" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B108" s="128" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="D108" s="10"/>
       <c r="E108" s="10" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="F108" s="116" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="109" spans="1:6" ht="25.5" customHeight="1">
       <c r="A109" s="102" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B109" s="57" t="s">
+        <v>704</v>
+      </c>
+      <c r="C109" s="33" t="s">
         <v>705</v>
       </c>
-      <c r="C109" s="33" t="s">
+      <c r="D109" s="33" t="s">
         <v>706</v>
-      </c>
-      <c r="D109" s="33" t="s">
-        <v>707</v>
       </c>
       <c r="E109" s="33" t="s">
         <v>534</v>
@@ -18365,27 +18383,27 @@
     </row>
     <row r="110" spans="1:6" ht="30" customHeight="1">
       <c r="A110" s="103" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B110" s="58" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C110" s="39" t="s">
-        <v>973</v>
+        <v>970</v>
       </c>
       <c r="D110" s="39" t="s">
-        <v>974</v>
+        <v>971</v>
       </c>
       <c r="E110" s="39" t="s">
         <v>534</v>
       </c>
       <c r="F110" s="118" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
     </row>
     <row r="111" spans="1:6" ht="25.5" customHeight="1">
       <c r="A111" s="155" t="s">
-        <v>980</v>
+        <v>977</v>
       </c>
       <c r="B111" s="156"/>
       <c r="C111" s="156"/>
@@ -18395,16 +18413,16 @@
     </row>
     <row r="112" spans="1:6" ht="42" customHeight="1">
       <c r="A112" s="101" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B112" s="56" t="s">
         <v>495</v>
       </c>
       <c r="C112" s="10" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D112" s="10" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="E112" s="10" t="s">
         <v>20</v>
@@ -18415,59 +18433,59 @@
     </row>
     <row r="113" spans="1:6" ht="45" customHeight="1">
       <c r="A113" s="105" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B113" s="60" t="s">
         <v>497</v>
       </c>
       <c r="C113" s="61" t="s">
+        <v>709</v>
+      </c>
+      <c r="D113" s="61" t="s">
         <v>710</v>
-      </c>
-      <c r="D113" s="61" t="s">
-        <v>711</v>
       </c>
       <c r="E113" s="61" t="s">
         <v>500</v>
       </c>
       <c r="F113" s="120" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="25.5" customHeight="1">
       <c r="A114" s="105" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B114" s="60" t="s">
+        <v>712</v>
+      </c>
+      <c r="C114" s="61" t="s">
         <v>713</v>
       </c>
-      <c r="C114" s="61" t="s">
+      <c r="D114" s="61" t="s">
         <v>714</v>
       </c>
-      <c r="D114" s="61" t="s">
+      <c r="E114" s="61" t="s">
         <v>715</v>
       </c>
-      <c r="E114" s="61" t="s">
+      <c r="F114" s="120" t="s">
         <v>716</v>
-      </c>
-      <c r="F114" s="120" t="s">
-        <v>717</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="21.75" customHeight="1">
       <c r="A115" s="105" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B115" s="60" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="C115" s="61" t="s">
+        <v>717</v>
+      </c>
+      <c r="D115" s="61" t="s">
         <v>718</v>
       </c>
-      <c r="D115" s="61" t="s">
+      <c r="E115" s="61" t="s">
         <v>719</v>
-      </c>
-      <c r="E115" s="61" t="s">
-        <v>720</v>
       </c>
       <c r="F115" s="120" t="s">
         <v>363</v>
@@ -18475,39 +18493,39 @@
     </row>
     <row r="116" spans="1:6" ht="25.5" customHeight="1">
       <c r="A116" s="105" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B116" s="207" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C116" s="61" t="s">
+        <v>943</v>
+      </c>
+      <c r="D116" s="61" t="s">
+        <v>944</v>
+      </c>
+      <c r="E116" s="61" t="s">
+        <v>945</v>
+      </c>
+      <c r="F116" s="120" t="s">
         <v>946</v>
-      </c>
-      <c r="D116" s="61" t="s">
-        <v>947</v>
-      </c>
-      <c r="E116" s="61" t="s">
-        <v>948</v>
-      </c>
-      <c r="F116" s="120" t="s">
-        <v>949</v>
       </c>
     </row>
     <row r="117" spans="1:6" ht="25.5" customHeight="1">
       <c r="A117" s="98" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B117" s="53" t="s">
+        <v>720</v>
+      </c>
+      <c r="C117" s="5" t="s">
         <v>721</v>
       </c>
-      <c r="C117" s="5" t="s">
+      <c r="D117" s="5" t="s">
         <v>722</v>
       </c>
-      <c r="D117" s="5" t="s">
+      <c r="E117" s="5" t="s">
         <v>723</v>
-      </c>
-      <c r="E117" s="5" t="s">
-        <v>724</v>
       </c>
       <c r="F117" s="86" t="s">
         <v>113</v>
@@ -18515,19 +18533,19 @@
     </row>
     <row r="118" spans="1:6" ht="30" customHeight="1">
       <c r="A118" s="102" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B118" s="57" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C118" s="33" t="s">
+        <v>724</v>
+      </c>
+      <c r="D118" s="33" t="s">
         <v>725</v>
       </c>
-      <c r="D118" s="33" t="s">
+      <c r="E118" s="33" t="s">
         <v>726</v>
-      </c>
-      <c r="E118" s="33" t="s">
-        <v>727</v>
       </c>
       <c r="F118" s="117" t="s">
         <v>277</v>
@@ -18535,36 +18553,36 @@
     </row>
     <row r="119" spans="1:6" ht="25.5" customHeight="1">
       <c r="A119" s="105" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B119" s="60" t="s">
+        <v>727</v>
+      </c>
+      <c r="C119" s="61" t="s">
         <v>728</v>
       </c>
-      <c r="C119" s="61" t="s">
+      <c r="D119" s="61" t="s">
         <v>729</v>
-      </c>
-      <c r="D119" s="61" t="s">
-        <v>730</v>
       </c>
       <c r="E119" s="61" t="s">
         <v>480</v>
       </c>
       <c r="F119" s="120" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="30" customHeight="1">
       <c r="A120" s="106" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B120" s="63" t="s">
+        <v>731</v>
+      </c>
+      <c r="C120" s="20" t="s">
         <v>732</v>
       </c>
-      <c r="C120" s="20" t="s">
+      <c r="D120" s="20" t="s">
         <v>733</v>
-      </c>
-      <c r="D120" s="20" t="s">
-        <v>734</v>
       </c>
       <c r="E120" s="20" t="s">
         <v>529</v>
@@ -18575,99 +18593,99 @@
     </row>
     <row r="121" spans="1:6" ht="25.5" customHeight="1">
       <c r="A121" s="109" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B121" s="65" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C121" s="42" t="s">
+        <v>734</v>
+      </c>
+      <c r="D121" s="42" t="s">
         <v>735</v>
       </c>
-      <c r="D121" s="42" t="s">
+      <c r="E121" s="42" t="s">
         <v>736</v>
-      </c>
-      <c r="E121" s="42" t="s">
-        <v>737</v>
       </c>
       <c r="F121" s="124" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="122" spans="1:6" ht="25.5" customHeight="1">
+    <row r="122" spans="1:6" ht="110" customHeight="1">
       <c r="A122" s="99" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B122" s="54" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="C122" s="15" t="s">
-        <v>739</v>
+        <v>1066</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>740</v>
+        <v>1067</v>
       </c>
       <c r="E122" s="15" t="s">
-        <v>537</v>
+        <v>1068</v>
       </c>
       <c r="F122" s="85" t="s">
-        <v>131</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="123" spans="1:6" ht="42" customHeight="1">
       <c r="A123" s="103" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B123" s="58" t="s">
+        <v>738</v>
+      </c>
+      <c r="C123" s="39" t="s">
+        <v>739</v>
+      </c>
+      <c r="D123" s="39" t="s">
+        <v>740</v>
+      </c>
+      <c r="E123" s="39" t="s">
         <v>741</v>
       </c>
-      <c r="C123" s="39" t="s">
-        <v>742</v>
-      </c>
-      <c r="D123" s="39" t="s">
-        <v>743</v>
-      </c>
-      <c r="E123" s="39" t="s">
-        <v>744</v>
-      </c>
       <c r="F123" s="118" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="124" spans="1:6" ht="30" customHeight="1">
       <c r="A124" s="101" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B124" s="56" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="C124" s="10" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="D124" s="10" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="E124" s="10" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="F124" s="116" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="125" spans="1:6" ht="28">
       <c r="A125" s="103" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B125" s="58" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C125" s="39" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="D125" s="39" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="E125" s="39" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F125" s="118" t="s">
         <v>351</v>
@@ -18675,47 +18693,47 @@
     </row>
     <row r="126" spans="1:6" ht="28">
       <c r="A126" s="103" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B126" s="58" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C126" s="39" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="D126" s="39" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="E126" s="39" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F126" s="118" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
     </row>
     <row r="127" spans="1:6" ht="31">
       <c r="A127" s="104" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B127" s="59" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C127" s="47" t="s">
-        <v>976</v>
+        <v>973</v>
       </c>
       <c r="D127" s="47" t="s">
-        <v>977</v>
+        <v>974</v>
       </c>
       <c r="E127" s="47" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F127" s="119" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
     </row>
     <row r="128" spans="1:6">
       <c r="A128" s="158" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="B128" s="159"/>
       <c r="C128" s="159"/>
@@ -18725,19 +18743,19 @@
     </row>
     <row r="129" spans="1:6" ht="28">
       <c r="A129" s="101" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B129" s="56" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="C129" s="10" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D129" s="10" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F129" s="116" t="s">
         <v>37</v>
@@ -18745,39 +18763,39 @@
     </row>
     <row r="130" spans="1:6" ht="28">
       <c r="A130" s="100" t="s">
+        <v>752</v>
+      </c>
+      <c r="B130" s="55" t="s">
         <v>755</v>
       </c>
-      <c r="B130" s="55" t="s">
+      <c r="C130" s="50" t="s">
+        <v>756</v>
+      </c>
+      <c r="D130" s="50" t="s">
+        <v>757</v>
+      </c>
+      <c r="E130" s="50" t="s">
+        <v>674</v>
+      </c>
+      <c r="F130" s="115" t="s">
         <v>758</v>
-      </c>
-      <c r="C130" s="50" t="s">
-        <v>759</v>
-      </c>
-      <c r="D130" s="50" t="s">
-        <v>760</v>
-      </c>
-      <c r="E130" s="50" t="s">
-        <v>675</v>
-      </c>
-      <c r="F130" s="115" t="s">
-        <v>761</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="28">
       <c r="A131" s="100" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B131" s="55" t="s">
+        <v>759</v>
+      </c>
+      <c r="C131" s="50" t="s">
+        <v>760</v>
+      </c>
+      <c r="D131" s="50" t="s">
+        <v>761</v>
+      </c>
+      <c r="E131" s="50" t="s">
         <v>762</v>
-      </c>
-      <c r="C131" s="50" t="s">
-        <v>763</v>
-      </c>
-      <c r="D131" s="50" t="s">
-        <v>764</v>
-      </c>
-      <c r="E131" s="50" t="s">
-        <v>765</v>
       </c>
       <c r="F131" s="115" t="s">
         <v>406</v>
@@ -18785,99 +18803,99 @@
     </row>
     <row r="132" spans="1:6" ht="28">
       <c r="A132" s="100" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B132" s="55" t="s">
+        <v>763</v>
+      </c>
+      <c r="C132" s="50" t="s">
+        <v>764</v>
+      </c>
+      <c r="D132" s="50" t="s">
+        <v>765</v>
+      </c>
+      <c r="E132" s="50" t="s">
         <v>766</v>
       </c>
-      <c r="C132" s="50" t="s">
+      <c r="F132" s="115" t="s">
         <v>767</v>
-      </c>
-      <c r="D132" s="50" t="s">
-        <v>768</v>
-      </c>
-      <c r="E132" s="50" t="s">
-        <v>769</v>
-      </c>
-      <c r="F132" s="115" t="s">
-        <v>770</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="28">
       <c r="A133" s="99" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B133" s="54" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="C133" s="15" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="D133" s="15" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="E133" s="15" t="s">
         <v>405</v>
       </c>
       <c r="F133" s="85" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
     </row>
     <row r="134" spans="1:6" ht="28">
       <c r="A134" s="98" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B134" s="53" t="s">
+        <v>771</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>772</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>773</v>
+      </c>
+      <c r="E134" s="5" t="s">
         <v>774</v>
       </c>
-      <c r="C134" s="5" t="s">
-        <v>775</v>
-      </c>
-      <c r="D134" s="5" t="s">
-        <v>776</v>
-      </c>
-      <c r="E134" s="5" t="s">
-        <v>777</v>
-      </c>
       <c r="F134" s="114" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
     </row>
     <row r="135" spans="1:6" ht="28">
       <c r="A135" s="99" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B135" s="54" t="s">
+        <v>775</v>
+      </c>
+      <c r="C135" s="15" t="s">
+        <v>776</v>
+      </c>
+      <c r="D135" s="15" t="s">
+        <v>777</v>
+      </c>
+      <c r="E135" s="15" t="s">
         <v>778</v>
       </c>
-      <c r="C135" s="15" t="s">
-        <v>779</v>
-      </c>
-      <c r="D135" s="15" t="s">
-        <v>780</v>
-      </c>
-      <c r="E135" s="15" t="s">
-        <v>781</v>
-      </c>
       <c r="F135" s="113" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="28">
       <c r="A136" s="98" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B136" s="53" t="s">
+        <v>779</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>781</v>
+      </c>
+      <c r="E136" s="5" t="s">
         <v>782</v>
-      </c>
-      <c r="C136" s="5" t="s">
-        <v>783</v>
-      </c>
-      <c r="D136" s="5" t="s">
-        <v>784</v>
-      </c>
-      <c r="E136" s="5" t="s">
-        <v>785</v>
       </c>
       <c r="F136" s="114" t="s">
         <v>254</v>
@@ -18885,22 +18903,22 @@
     </row>
     <row r="137" spans="1:6" ht="29" thickBot="1">
       <c r="A137" s="112" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B137" s="96" t="s">
         <v>492</v>
       </c>
       <c r="C137" s="97" t="s">
+        <v>783</v>
+      </c>
+      <c r="D137" s="97" t="s">
+        <v>784</v>
+      </c>
+      <c r="E137" s="97" t="s">
+        <v>785</v>
+      </c>
+      <c r="F137" s="127" t="s">
         <v>786</v>
-      </c>
-      <c r="D137" s="97" t="s">
-        <v>787</v>
-      </c>
-      <c r="E137" s="97" t="s">
-        <v>788</v>
-      </c>
-      <c r="F137" s="127" t="s">
-        <v>789</v>
       </c>
     </row>
   </sheetData>
@@ -18926,7 +18944,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -19027,7 +19045,7 @@
         <v>62</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="C8" s="17" t="s">
         <v>64</v>
@@ -19044,13 +19062,13 @@
         <v>53</v>
       </c>
       <c r="B9" s="69" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="C9" s="67" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="D9" s="66" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="E9" s="68" t="s">
         <v>184</v>
@@ -19061,13 +19079,13 @@
         <v>53</v>
       </c>
       <c r="B10" s="69" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="C10" s="67" t="s">
         <v>206</v>
       </c>
       <c r="D10" s="66" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="E10" s="68" t="s">
         <v>61</v>
@@ -19112,30 +19130,30 @@
         <v>67</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>1046</v>
+        <v>1043</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>1041</v>
+        <v>1038</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>1048</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="42" customHeight="1">
       <c r="A14" s="20" t="s">
-        <v>1049</v>
+        <v>1046</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>1045</v>
+        <v>1042</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>1051</v>
+        <v>1048</v>
       </c>
       <c r="E14" s="23" t="s">
         <v>71</v>
@@ -19143,19 +19161,19 @@
     </row>
     <row r="15" spans="1:5" ht="56" customHeight="1">
       <c r="A15" s="20" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E15" s="23" t="s">
         <v>1057</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>1058</v>
-      </c>
-      <c r="C15" s="22" t="s">
-        <v>1056</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>1059</v>
-      </c>
-      <c r="E15" s="23" t="s">
-        <v>1060</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="70" customHeight="1">
@@ -19163,16 +19181,16 @@
         <v>90</v>
       </c>
       <c r="B16" s="20" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>1063</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>1064</v>
+      </c>
+      <c r="E16" s="23" t="s">
         <v>1065</v>
-      </c>
-      <c r="C16" s="22" t="s">
-        <v>1066</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>1067</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>1068</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1"/>
@@ -19292,13 +19310,13 @@
         <v>90</v>
       </c>
       <c r="B25" s="66" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="C25" s="67" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="D25" s="66" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="E25" s="68" t="s">
         <v>234</v>
@@ -19489,13 +19507,13 @@
         <v>67</v>
       </c>
       <c r="B38" s="73" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="C38" s="71" t="s">
         <v>271</v>
       </c>
       <c r="D38" s="70" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="E38" s="72" t="s">
         <v>103</v>
@@ -19516,6 +19534,23 @@
       </c>
       <c r="E39" s="23" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="110" customHeight="1">
+      <c r="A40" s="20" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C40" s="22" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D40" s="20" t="s">
+        <v>1073</v>
+      </c>
+      <c r="E40" s="23" t="s">
+        <v>1074</v>
       </c>
     </row>
   </sheetData>
@@ -19548,7 +19583,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1">
       <c r="A1" s="191" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
       <c r="B1" s="192"/>
       <c r="C1" s="192"/>
@@ -19558,7 +19593,7 @@
     </row>
     <row r="2" spans="1:6" ht="45" customHeight="1">
       <c r="A2" s="194" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="B2" s="195"/>
       <c r="C2" s="195"/>
@@ -19658,19 +19693,19 @@
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1">
       <c r="A8" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B8" s="75">
         <v>4.5</v>
       </c>
       <c r="C8" s="76" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="D8" s="75" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="E8" s="76" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="F8" s="87" t="s">
         <v>152</v>
@@ -19678,19 +19713,19 @@
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1">
       <c r="A9" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B9" s="68">
         <v>4.5</v>
       </c>
       <c r="C9" s="66" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="D9" s="68" t="s">
         <v>107</v>
       </c>
       <c r="E9" s="66" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="F9" s="88" t="s">
         <v>152</v>
@@ -19720,7 +19755,7 @@
         <v>57</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
       <c r="F11" s="84" t="s">
         <v>164</v>
@@ -19768,59 +19803,59 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1">
       <c r="A14" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B14" s="75">
         <v>4.8</v>
       </c>
       <c r="C14" s="76" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="D14" s="75" t="s">
         <v>66</v>
       </c>
       <c r="E14" s="76" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="F14" s="87" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="30" customHeight="1">
       <c r="A15" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B15" s="68">
         <v>4.5999999999999996</v>
       </c>
       <c r="C15" s="66" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="D15" s="68" t="s">
         <v>111</v>
       </c>
       <c r="E15" s="66" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="F15" s="88" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1">
       <c r="A16" s="82" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="B16" s="216" t="s">
-        <v>1028</v>
+        <v>1025</v>
       </c>
       <c r="C16" s="66" t="s">
-        <v>1029</v>
+        <v>1026</v>
       </c>
       <c r="D16" s="68" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="E16" s="66" t="s">
-        <v>1030</v>
+        <v>1027</v>
       </c>
       <c r="F16" s="88" t="s">
         <v>477</v>
@@ -19828,22 +19863,22 @@
     </row>
     <row r="17" spans="1:6" ht="30" customHeight="1">
       <c r="A17" s="82" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="B17" s="216" t="s">
-        <v>1031</v>
+        <v>1028</v>
       </c>
       <c r="C17" s="66" t="s">
-        <v>1032</v>
+        <v>1029</v>
       </c>
       <c r="D17" s="68" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
       <c r="E17" s="66" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="F17" s="88" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="30" customHeight="1">
@@ -19924,13 +19959,13 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="C22" s="76" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="D22" s="75" t="s">
         <v>256</v>
       </c>
       <c r="E22" s="76" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
       <c r="F22" s="87" t="s">
         <v>301</v>
@@ -19938,22 +19973,22 @@
     </row>
     <row r="23" spans="1:6" ht="30" customHeight="1">
       <c r="A23" s="82" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B23" s="68">
         <v>4.3</v>
       </c>
       <c r="C23" s="66" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="D23" s="68" t="s">
         <v>256</v>
       </c>
       <c r="E23" s="66" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="F23" s="88" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="30" customHeight="1">
@@ -20028,42 +20063,42 @@
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1">
       <c r="A28" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B28" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C28" s="76" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="D28" s="75" t="s">
         <v>160</v>
       </c>
       <c r="E28" s="76" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="F28" s="87" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="30" customHeight="1">
       <c r="A29" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B29" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C29" s="66" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="D29" s="68" t="s">
         <v>219</v>
       </c>
       <c r="E29" s="66" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="F29" s="88" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="30" customHeight="1">
@@ -20124,33 +20159,33 @@
         <v>4.3</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="F33" s="86" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="19.5" customHeight="1">
       <c r="A34" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B34" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C34" s="76" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="D34" s="75" t="s">
         <v>166</v>
       </c>
       <c r="E34" s="76" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="F34" s="87" t="s">
         <v>206</v>
@@ -20158,22 +20193,22 @@
     </row>
     <row r="35" spans="1:6" ht="30" customHeight="1">
       <c r="A35" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B35" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C35" s="66" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="D35" s="68" t="s">
         <v>61</v>
       </c>
       <c r="E35" s="66" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="F35" s="88" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="30" customHeight="1">
@@ -20194,16 +20229,16 @@
         <v>4.5</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>877</v>
+        <v>874</v>
       </c>
       <c r="D37" s="27" t="s">
         <v>219</v>
       </c>
       <c r="E37" s="28" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
       <c r="F37" s="84" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="30" customHeight="1">
@@ -20248,19 +20283,19 @@
     </row>
     <row r="40" spans="1:6" ht="19.5" customHeight="1">
       <c r="A40" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B40" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C40" s="76" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
       <c r="D40" s="75" t="s">
         <v>215</v>
       </c>
       <c r="E40" s="76" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
       <c r="F40" s="87" t="s">
         <v>92</v>
@@ -20268,19 +20303,19 @@
     </row>
     <row r="41" spans="1:6" ht="30" customHeight="1">
       <c r="A41" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B41" s="68">
         <v>4.3</v>
       </c>
       <c r="C41" s="66" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
       <c r="D41" s="68" t="s">
         <v>223</v>
       </c>
       <c r="E41" s="66" t="s">
-        <v>851</v>
+        <v>848</v>
       </c>
       <c r="F41" s="88" t="s">
         <v>92</v>
@@ -20358,19 +20393,19 @@
     </row>
     <row r="46" spans="1:6" ht="19.5" customHeight="1">
       <c r="A46" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B46" s="75">
         <v>4.5</v>
       </c>
       <c r="C46" s="76" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="D46" s="75" t="s">
         <v>89</v>
       </c>
       <c r="E46" s="76" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="F46" s="87" t="s">
         <v>225</v>
@@ -20378,22 +20413,22 @@
     </row>
     <row r="47" spans="1:6" ht="30" customHeight="1">
       <c r="A47" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B47" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C47" s="66" t="s">
+        <v>817</v>
+      </c>
+      <c r="D47" s="68" t="s">
+        <v>818</v>
+      </c>
+      <c r="E47" s="66" t="s">
+        <v>819</v>
+      </c>
+      <c r="F47" s="88" t="s">
         <v>820</v>
-      </c>
-      <c r="D47" s="68" t="s">
-        <v>821</v>
-      </c>
-      <c r="E47" s="66" t="s">
-        <v>822</v>
-      </c>
-      <c r="F47" s="88" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="30" customHeight="1">
@@ -20454,56 +20489,56 @@
         <v>4.5</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>867</v>
+        <v>864</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>219</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
       <c r="F51" s="86" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="19.5" customHeight="1">
       <c r="A52" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B52" s="75">
         <v>4.7</v>
       </c>
       <c r="C52" s="76" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="D52" s="75" t="s">
         <v>66</v>
       </c>
       <c r="E52" s="76" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="F52" s="87" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="30" customHeight="1">
       <c r="A53" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B53" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C53" s="66" t="s">
+        <v>824</v>
+      </c>
+      <c r="D53" s="68" t="s">
+        <v>825</v>
+      </c>
+      <c r="E53" s="66" t="s">
+        <v>826</v>
+      </c>
+      <c r="F53" s="88" t="s">
         <v>827</v>
-      </c>
-      <c r="D53" s="68" t="s">
-        <v>828</v>
-      </c>
-      <c r="E53" s="66" t="s">
-        <v>829</v>
-      </c>
-      <c r="F53" s="88" t="s">
-        <v>830</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="30" customHeight="1">
@@ -20578,42 +20613,42 @@
     </row>
     <row r="58" spans="1:6" ht="19.5" customHeight="1">
       <c r="A58" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B58" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C58" s="74" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="D58" s="75" t="s">
         <v>219</v>
       </c>
       <c r="E58" s="76" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="F58" s="87" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="30" customHeight="1">
       <c r="A59" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B59" s="68">
         <v>4.5999999999999996</v>
       </c>
       <c r="C59" s="69" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="D59" s="68" t="s">
         <v>52</v>
       </c>
       <c r="E59" s="66" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="F59" s="88" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="30" customHeight="1">
@@ -20710,7 +20745,7 @@
         <v>115</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>1035</v>
+        <v>1032</v>
       </c>
       <c r="F65" s="84" t="s">
         <v>113</v>
@@ -20724,13 +20759,13 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="C66" s="16" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="D66" s="18" t="s">
         <v>223</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
       <c r="F66" s="85" t="s">
         <v>277</v>
@@ -20758,19 +20793,19 @@
     </row>
     <row r="68" spans="1:6" ht="30" customHeight="1">
       <c r="A68" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B68" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C68" s="76" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="D68" s="75" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="E68" s="76" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="F68" s="87" t="s">
         <v>277</v>
@@ -20778,39 +20813,39 @@
     </row>
     <row r="69" spans="1:6" ht="30" customHeight="1">
       <c r="A69" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B69" s="68">
         <v>4.3</v>
       </c>
       <c r="C69" s="66" t="s">
+        <v>870</v>
+      </c>
+      <c r="D69" s="68" t="s">
+        <v>871</v>
+      </c>
+      <c r="E69" s="66" t="s">
+        <v>872</v>
+      </c>
+      <c r="F69" s="88" t="s">
         <v>873</v>
-      </c>
-      <c r="D69" s="68" t="s">
-        <v>874</v>
-      </c>
-      <c r="E69" s="66" t="s">
-        <v>875</v>
-      </c>
-      <c r="F69" s="88" t="s">
-        <v>876</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="30" customHeight="1">
       <c r="A70" s="81" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="B70" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C70" s="76" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="D70" s="75" t="s">
         <v>123</v>
       </c>
       <c r="E70" s="76" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="F70" s="87" t="s">
         <v>121</v>
@@ -20818,39 +20853,39 @@
     </row>
     <row r="71" spans="1:6" ht="30" customHeight="1">
       <c r="A71" s="82" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="B71" s="68">
         <v>4.5</v>
       </c>
       <c r="C71" s="66" t="s">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="D71" s="68" t="s">
         <v>99</v>
       </c>
       <c r="E71" s="66" t="s">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="F71" s="88" t="s">
-        <v>895</v>
+        <v>892</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="30" customHeight="1">
       <c r="A72" s="82" t="s">
-        <v>1010</v>
+        <v>1007</v>
       </c>
       <c r="B72" s="216" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C72" s="66" t="s">
+        <v>1018</v>
+      </c>
+      <c r="D72" s="68" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E72" s="66" t="s">
         <v>1020</v>
-      </c>
-      <c r="C72" s="66" t="s">
-        <v>1021</v>
-      </c>
-      <c r="D72" s="68" t="s">
-        <v>1022</v>
-      </c>
-      <c r="E72" s="66" t="s">
-        <v>1023</v>
       </c>
       <c r="F72" s="88" t="s">
         <v>288</v>
@@ -20858,22 +20893,22 @@
     </row>
     <row r="73" spans="1:6" ht="30" customHeight="1">
       <c r="A73" s="82" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B73" s="216" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C73" s="66" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D73" s="68" t="s">
         <v>1014</v>
       </c>
-      <c r="B73" s="216" t="s">
+      <c r="E73" s="66" t="s">
+        <v>1023</v>
+      </c>
+      <c r="F73" s="88" t="s">
         <v>1024</v>
-      </c>
-      <c r="C73" s="66" t="s">
-        <v>1025</v>
-      </c>
-      <c r="D73" s="68" t="s">
-        <v>1017</v>
-      </c>
-      <c r="E73" s="66" t="s">
-        <v>1026</v>
-      </c>
-      <c r="F73" s="88" t="s">
-        <v>1027</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="30" customHeight="1">
@@ -20948,19 +20983,19 @@
     </row>
     <row r="78" spans="1:6" ht="30" customHeight="1">
       <c r="A78" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B78" s="75">
         <v>4.3</v>
       </c>
       <c r="C78" s="76" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
       <c r="D78" s="75" t="s">
         <v>219</v>
       </c>
       <c r="E78" s="76" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="F78" s="87" t="s">
         <v>271</v>
@@ -20968,19 +21003,19 @@
     </row>
     <row r="79" spans="1:6" ht="30" customHeight="1">
       <c r="A79" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B79" s="68">
         <v>4</v>
       </c>
       <c r="C79" s="66" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="D79" s="68" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="E79" s="66" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="F79" s="88" t="s">
         <v>271</v>
@@ -21024,13 +21059,13 @@
         <v>4.2</v>
       </c>
       <c r="C82" s="16" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="D82" s="18" t="s">
         <v>119</v>
       </c>
       <c r="E82" s="15" t="s">
-        <v>858</v>
+        <v>855</v>
       </c>
       <c r="F82" s="85" t="s">
         <v>277</v>
@@ -21044,13 +21079,13 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="C83" s="13" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>219</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>881</v>
+        <v>878</v>
       </c>
       <c r="F83" s="86" t="s">
         <v>277</v>
@@ -21058,19 +21093,19 @@
     </row>
     <row r="84" spans="1:6" ht="30" customHeight="1">
       <c r="A84" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B84" s="75">
         <v>4.3</v>
       </c>
       <c r="C84" s="76" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
       <c r="D84" s="75" t="s">
         <v>119</v>
       </c>
       <c r="E84" s="76" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="F84" s="87" t="s">
         <v>277</v>
@@ -21078,19 +21113,19 @@
     </row>
     <row r="85" spans="1:6" ht="30" customHeight="1">
       <c r="A85" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B85" s="68">
         <v>4.4000000000000004</v>
       </c>
       <c r="C85" s="66" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="D85" s="68" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="E85" s="66" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="F85" s="88" t="s">
         <v>288</v>
@@ -21098,19 +21133,19 @@
     </row>
     <row r="86" spans="1:6" ht="30" customHeight="1">
       <c r="A86" s="81" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="B86" s="75">
         <v>4.5999999999999996</v>
       </c>
       <c r="C86" s="76" t="s">
-        <v>896</v>
+        <v>893</v>
       </c>
       <c r="D86" s="75" t="s">
         <v>128</v>
       </c>
       <c r="E86" s="76" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
       <c r="F86" s="87" t="s">
         <v>277</v>
@@ -21118,19 +21153,19 @@
     </row>
     <row r="87" spans="1:6" ht="30" customHeight="1">
       <c r="A87" s="82" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="B87" s="68" t="s">
         <v>254</v>
       </c>
       <c r="C87" s="66" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="D87" s="68" t="s">
         <v>289</v>
       </c>
       <c r="E87" s="66" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="F87" s="88" t="s">
         <v>113</v>
@@ -21138,19 +21173,19 @@
     </row>
     <row r="88" spans="1:6" ht="30" customHeight="1">
       <c r="A88" s="82" t="s">
-        <v>1010</v>
+        <v>1007</v>
       </c>
       <c r="B88" s="216" t="s">
-        <v>1011</v>
+        <v>1008</v>
       </c>
       <c r="C88" s="66" t="s">
-        <v>1012</v>
+        <v>1009</v>
       </c>
       <c r="D88" s="68" t="s">
         <v>189</v>
       </c>
       <c r="E88" s="66" t="s">
-        <v>1013</v>
+        <v>1010</v>
       </c>
       <c r="F88" s="88" t="s">
         <v>264</v>
@@ -21158,22 +21193,22 @@
     </row>
     <row r="89" spans="1:6" ht="30" customHeight="1">
       <c r="A89" s="82" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B89" s="216" t="s">
+        <v>1012</v>
+      </c>
+      <c r="C89" s="66" t="s">
+        <v>1013</v>
+      </c>
+      <c r="D89" s="68" t="s">
         <v>1014</v>
       </c>
-      <c r="B89" s="216" t="s">
+      <c r="E89" s="66" t="s">
         <v>1015</v>
       </c>
-      <c r="C89" s="66" t="s">
+      <c r="F89" s="88" t="s">
         <v>1016</v>
-      </c>
-      <c r="D89" s="68" t="s">
-        <v>1017</v>
-      </c>
-      <c r="E89" s="66" t="s">
-        <v>1018</v>
-      </c>
-      <c r="F89" s="88" t="s">
-        <v>1019</v>
       </c>
     </row>
     <row r="90" spans="1:6" ht="33.75" customHeight="1">
@@ -21248,39 +21283,39 @@
     </row>
     <row r="94" spans="1:6" ht="28">
       <c r="A94" s="81" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B94" s="75">
         <v>4.4000000000000004</v>
       </c>
       <c r="C94" s="76" t="s">
+        <v>882</v>
+      </c>
+      <c r="D94" s="75" t="s">
+        <v>883</v>
+      </c>
+      <c r="E94" s="76" t="s">
+        <v>884</v>
+      </c>
+      <c r="F94" s="87" t="s">
         <v>885</v>
-      </c>
-      <c r="D94" s="75" t="s">
-        <v>886</v>
-      </c>
-      <c r="E94" s="76" t="s">
-        <v>887</v>
-      </c>
-      <c r="F94" s="87" t="s">
-        <v>888</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="28">
       <c r="A95" s="82" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="B95" s="68">
         <v>4.5</v>
       </c>
       <c r="C95" s="66" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="D95" s="68" t="s">
         <v>119</v>
       </c>
       <c r="E95" s="66" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="F95" s="88" t="s">
         <v>278</v>
@@ -21288,7 +21323,7 @@
     </row>
     <row r="96" spans="1:6" ht="48" customHeight="1" thickBot="1">
       <c r="A96" s="182" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="B96" s="183"/>
       <c r="C96" s="183"/>
@@ -21446,13 +21481,13 @@
         <v>324</v>
       </c>
       <c r="B10" s="92" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="C10" s="92" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="D10" s="125" t="s">
-        <v>931</v>
+        <v>928</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -21572,27 +21607,27 @@
         <v>324</v>
       </c>
       <c r="B20" s="92" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="C20" s="92" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="D20" s="125" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="30" customHeight="1">
       <c r="A21" s="140" t="s">
+        <v>932</v>
+      </c>
+      <c r="B21" s="90" t="s">
+        <v>933</v>
+      </c>
+      <c r="C21" s="90" t="s">
+        <v>934</v>
+      </c>
+      <c r="D21" s="149" t="s">
         <v>935</v>
-      </c>
-      <c r="B21" s="90" t="s">
-        <v>936</v>
-      </c>
-      <c r="C21" s="90" t="s">
-        <v>937</v>
-      </c>
-      <c r="D21" s="149" t="s">
-        <v>938</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="27.75" customHeight="1">

</xml_diff>